<commit_message>
Delete the form TC-FORM-004 creates when the server wrongly accepts a blank name
The real server answers 201 to a form create with name "" and the form exists whatever
the assertion says. The test now registers the response for cleanup before asserting
(register_created_form), and the end-of-run cleanup deletes every registered form right
after the run's own form and before the crop variety (it references the variety too):
one DELETE and one "form (TC-FORM-004 blank name)" row in the report's Cleanup section
each; nothing runs when the request is refused.

Catalogue: new TC-CLEANUP-004 row (later cleanup rows renumbered 005-009), TC-FORM-004
description updated; README updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cropin_API_Test_Scenarios.xlsx
+++ b/docs/Cropin_API_Test_Scenarios.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E115"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>100 test scenarios across auth/farmer/asset/plantype/crop_variety/plan/project, task fill, form, the cleanup teardown chain, and the intake-validation framework self-tests</t>
+          <t>101 test scenarios across auth/farmer/asset/plantype/crop_variety/plan/project, task fill, form, the cleanup teardown chain, and the intake-validation framework self-tests</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>(`test_create_form_blank_name_rejected`) Negative: the normal create body (shared crop variety) with name "" is rejected with a 4xx (not a server error) and the response carries no new form id. The exact code is frozen in test data (form.expectations) after the first real run; a 2xx fails the test.</t>
+          <t>(`test_create_form_blank_name_rejected`) Negative: the normal create body (shared crop variety) with name "" is rejected with a 4xx (not a server error) and the response carries no new form id. A 2xx fails the test (the real server does accept a blank name) — and the form it created is still registered for cleanup and deleted at the end (TC-CLEANUP-004).</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Cleanup - Delete Crop Variety</t>
+          <t>Cleanup - Delete Forms Created By Negative Tests</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
@@ -2895,12 +2895,12 @@
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>(`cleanup_delete_crop_variety`) Deletes the shared crop variety created this run. Runs after the plan and form deletes, since both reference it.</t>
+          <t>(`cleanup_delete_extra_forms`) Deletes any form a test created by accident: when the server wrongly accepts the blank-name create of TC-FORM-004 (201), that form exists whatever the assertion says, so it is registered for cleanup before the assertion and deleted here, right after the shared form and before the crop variety (it references the variety too). One DELETE and one report row per such form; nothing runs when the request was refused. Judged like the form delete: its id must be in deletedIds.</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>DELETE /services/farm/api/varieties/bulk?ids=...</t>
+          <t>DELETE /services/form/api/forms/bulk?ids={id}</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Cleanup - Delete Asset</t>
+          <t>Cleanup - Delete Crop Variety</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
@@ -2922,12 +2922,12 @@
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>(`cleanup_delete_asset`) Deletes the shared asset created this run.</t>
+          <t>(`cleanup_delete_crop_variety`) Deletes the shared crop variety created this run. Runs after the plan and form deletes, since both reference it.</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>DELETE /services/farm/api/assets/bulk?ids=...</t>
+          <t>DELETE /services/farm/api/varieties/bulk?ids=...</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>Cleanup - Delete Farmer</t>
+          <t>Cleanup - Delete Asset</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>(`cleanup_delete_farmer`) Deletes the shared farmer created this run.</t>
+          <t>(`cleanup_delete_asset`) Deletes the shared asset created this run.</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>DELETE /services/farm/api/farmers/bulk?ids=...</t>
+          <t>DELETE /services/farm/api/assets/bulk?ids=...</t>
         </is>
       </c>
     </row>
@@ -2966,100 +2966,100 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
+          <t>Cleanup - Delete Farmer</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>(`cleanup_delete_farmer`) Deletes the shared farmer created this run.</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>DELETE /services/farm/api/farmers/bulk?ids=...</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>TC-CLEANUP-008</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
           <t>Cleanup - Stop Project Execution</t>
         </is>
       </c>
-      <c r="C99" s="8" t="inlineStr">
+      <c r="C100" s="8" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
       </c>
-      <c r="D99" s="7" t="inlineStr">
+      <c r="D100" s="7" t="inlineStr">
         <is>
           <t>(`cleanup_stop_project_execution`) Stops the shared project's execution — an async job, polled to completion — required before the project's other records can be considered fully torn down.</t>
         </is>
       </c>
-      <c r="E99" s="7" t="inlineStr">
+      <c r="E100" s="7" t="inlineStr">
         <is>
           <t>POST /services/farm/api/projects/{id}/stop-execution
 GET /services/farm/api/bulk-process/{job_id} (polled)</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="6" t="inlineStr">
-        <is>
-          <t>TC-CLEANUP-008</t>
-        </is>
-      </c>
-      <c r="B100" s="7" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>TC-CLEANUP-009</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
         <is>
           <t>Cleanup - Delete Plan Type</t>
         </is>
       </c>
-      <c r="C100" s="8" t="inlineStr">
+      <c r="C101" s="8" t="inlineStr">
         <is>
           <t>Cleanup</t>
         </is>
       </c>
-      <c r="D100" s="7" t="inlineStr">
+      <c r="D101" s="7" t="inlineStr">
         <is>
           <t>(`cleanup_delete_plan_type`) Deletes the shared plan type created this run. Last step of the whole teardown chain, run only once every other record above is already gone.</t>
         </is>
       </c>
-      <c r="E100" s="7" t="inlineStr">
+      <c r="E101" s="7" t="inlineStr">
         <is>
           <t>DELETE /services/farm/api/plan-types/bulk?ids=...</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="4" t="inlineStr">
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>FRAMEWORK (Intake Validation, Report Email)</t>
         </is>
       </c>
-      <c r="B101" s="5" t="n"/>
-      <c r="C101" s="5" t="n"/>
-      <c r="D101" s="5" t="n"/>
-      <c r="E101" s="5" t="n"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="6" t="inlineStr">
-        <is>
-          <t>TC-FW-001</t>
-        </is>
-      </c>
-      <c r="B102" s="7" t="inlineStr">
-        <is>
-          <t>Intake Spec - Valid Spec Accepted</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t>N/A (no marker)</t>
-        </is>
-      </c>
-      <c r="D102" s="7" t="inlineStr">
-        <is>
-          <t>(`test_valid_spec_passes`) Verifies a fully valid single-scenario intake spec passes schema validation.</t>
-        </is>
-      </c>
-      <c r="E102" s="7" t="inlineStr">
-        <is>
-          <t>N/A (unit test, no live API call)</t>
-        </is>
-      </c>
+      <c r="B102" s="5" t="n"/>
+      <c r="C102" s="5" t="n"/>
+      <c r="D102" s="5" t="n"/>
+      <c r="E102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-002</t>
+          <t>TC-FW-001</t>
         </is>
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Unknown Module Rejected</t>
+          <t>Intake Spec - Valid Spec Accepted</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>(`test_unknown_module_rejected`) Verifies an intake spec naming a module outside the allowed set (farmer/asset/plantype/crop_variety/project/login) is rejected.</t>
+          <t>(`test_valid_spec_passes`) Verifies a fully valid single-scenario intake spec passes schema validation.</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
@@ -3081,12 +3081,12 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-003</t>
+          <t>TC-FW-002</t>
         </is>
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Unsupported Method Rejected</t>
+          <t>Intake Spec - Unknown Module Rejected</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>(`test_unsupported_method_rejected`) Verifies an intake spec using an HTTP method outside the allowed set is rejected.</t>
+          <t>(`test_unknown_module_rejected`) Verifies an intake spec naming a module outside the allowed set (farmer/asset/plantype/crop_variety/project/login) is rejected.</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
@@ -3108,12 +3108,12 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-004</t>
+          <t>TC-FW-003</t>
         </is>
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Unknown Test Type Rejected</t>
+          <t>Intake Spec - Unsupported Method Rejected</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>(`test_unknown_test_type_rejected`) Verifies an intake spec with a test_type outside sanity/smoke/regression is rejected.</t>
+          <t>(`test_unsupported_method_rejected`) Verifies an intake spec using an HTTP method outside the allowed set is rejected.</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
@@ -3135,12 +3135,12 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-005</t>
+          <t>TC-FW-004</t>
         </is>
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Endpoint Must Be Relative Path</t>
+          <t>Intake Spec - Unknown Test Type Rejected</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
@@ -3150,7 +3150,7 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>(`test_endpoint_must_be_relative_path`) Verifies an intake spec whose endpoint doesn't start with "/" is rejected.</t>
+          <t>(`test_unknown_test_type_rejected`) Verifies an intake spec with a test_type outside sanity/smoke/regression is rejected.</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
@@ -3162,12 +3162,12 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-006</t>
+          <t>TC-FW-005</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Body Method Without Payload Rejected</t>
+          <t>Intake Spec - Endpoint Must Be Relative Path</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>(`test_body_method_without_payload_rejected`) Verifies a POST/PUT/PATCH intake spec with an empty payload is rejected.</t>
+          <t>(`test_endpoint_must_be_relative_path`) Verifies an intake spec whose endpoint doesn't start with "/" is rejected.</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
@@ -3189,12 +3189,12 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-007</t>
+          <t>TC-FW-006</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - GET Without Payload Accepted</t>
+          <t>Intake Spec - Body Method Without Payload Rejected</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
@@ -3204,7 +3204,7 @@
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>(`test_get_without_payload_is_fine`) Verifies a GET intake spec with no payload is accepted, since payload is optional for GET.</t>
+          <t>(`test_body_method_without_payload_rejected`) Verifies a POST/PUT/PATCH intake spec with an empty payload is rejected.</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
@@ -3216,12 +3216,12 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-008</t>
+          <t>TC-FW-007</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Negative Scenario Requires Error Status</t>
+          <t>Intake Spec - GET Without Payload Accepted</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>(`test_negative_scenario_requires_error_status`) Verifies an intake spec marked negative:true but with a non-error expected_status is rejected.</t>
+          <t>(`test_get_without_payload_is_fine`) Verifies a GET intake spec with no payload is accepted, since payload is optional for GET.</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
@@ -3243,12 +3243,12 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-009</t>
+          <t>TC-FW-008</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Negative Scenario With Error Status Accepted</t>
+          <t>Intake Spec - Negative Scenario Requires Error Status</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>(`test_negative_scenario_with_error_status_passes`) Verifies an intake spec marked negative:true with a proper &gt;=400 expected_status is accepted.</t>
+          <t>(`test_negative_scenario_requires_error_status`) Verifies an intake spec marked negative:true but with a non-error expected_status is rejected.</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
@@ -3270,12 +3270,12 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-010</t>
+          <t>TC-FW-009</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Batch Validates All Items</t>
+          <t>Intake Spec - Negative Scenario With Error Status Accepted</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>(`test_batch_validates_all_items`) Verifies a batch of several valid intake specs all validate together successfully.</t>
+          <t>(`test_negative_scenario_with_error_status_passes`) Verifies an intake spec marked negative:true with a proper &gt;=400 expected_status is accepted.</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
@@ -3297,12 +3297,12 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-011</t>
+          <t>TC-FW-010</t>
         </is>
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Intake Spec - Batch Rejects Invalid Item</t>
+          <t>Intake Spec - Batch Validates All Items</t>
         </is>
       </c>
       <c r="C112" s="8" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>(`test_batch_rejects_if_any_item_invalid`) Verifies that if one scenario in an intake batch is invalid, validation of the whole batch fails.</t>
+          <t>(`test_batch_validates_all_items`) Verifies a batch of several valid intake specs all validate together successfully.</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
@@ -3324,12 +3324,12 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-012</t>
+          <t>TC-FW-011</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Report Email - Summary With No Failures</t>
+          <t>Intake Spec - Batch Rejects Invalid Item</t>
         </is>
       </c>
       <c r="C113" s="8" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>(`test_summary_with_no_failures_says_so`) Verifies the email result block reports how many tests ran, passed, failed (0), errored and were skipped, and says there are no failed test cases.</t>
+          <t>(`test_batch_rejects_if_any_item_invalid`) Verifies that if one scenario in an intake batch is invalid, validation of the whole batch fails.</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
@@ -3351,12 +3351,12 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>TC-FW-013</t>
+          <t>TC-FW-012</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>Report Email - Summary Lists Failed Tests</t>
+          <t>Report Email - Summary With No Failures</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>(`test_summary_lists_each_failed_test_with_the_count`) Verifies the email result block gives the failed-test count and lists each failed test case by name with the first line of why it failed (passed tests are not listed).</t>
+          <t>(`test_summary_with_no_failures_says_so`) Verifies the email result block reports how many tests ran, passed, failed (0), errored and were skipped, and says there are no failed test cases.</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
@@ -3378,25 +3378,52 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
+          <t>TC-FW-013</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>Report Email - Summary Lists Failed Tests</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>N/A (no marker)</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>(`test_summary_lists_each_failed_test_with_the_count`) Verifies the email result block gives the failed-test count and lists each failed test case by name with the first line of why it failed (passed tests are not listed).</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>N/A (unit test, no live API call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
           <t>TC-FW-014</t>
         </is>
       </c>
-      <c r="B115" s="7" t="inlineStr">
+      <c r="B116" s="7" t="inlineStr">
         <is>
           <t>Report Email - Summary Errors, Expected Failures And Long Reasons</t>
         </is>
       </c>
-      <c r="C115" s="8" t="inlineStr">
+      <c r="C116" s="8" t="inlineStr">
         <is>
           <t>N/A (no marker)</t>
         </is>
       </c>
-      <c r="D115" s="7" t="inlineStr">
+      <c r="D116" s="7" t="inlineStr">
         <is>
           <t>(`test_summary_counts_errors_and_expected_failures_separately_and_shortens_long_reasons`) Verifies setup/teardown errors are counted and listed apart from failures, expected failures (xfail) are counted but not listed as failures, and very long failure reasons are shortened.</t>
         </is>
       </c>
-      <c r="E115" s="7" t="inlineStr">
+      <c r="E116" s="7" t="inlineStr">
         <is>
           <t>N/A (unit test, no live API call)</t>
         </is>
@@ -3412,7 +3439,7 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A86:E86"/>
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A101:E101"/>
+    <mergeCell ref="A102:E102"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A18:E18"/>

</xml_diff>